<commit_message>
feat: add client_type field (DEVELOPER/ENDUSER/ผู้รับเหมา)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/TEMPLATE_ลูกค้า.xlsx
+++ b/public/templates/TEMPLATE_ลูกค้า.xlsx
@@ -397,16 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:F5"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="22.83203125" customWidth="1"/>
     <col min="5" max="5" width="22.83203125" customWidth="1"/>
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,13 +424,7 @@
         <v>อีเมล</v>
       </c>
       <c r="F1" t="str">
-        <v>ที่อยู่</v>
-      </c>
-      <c r="G1" t="str">
-        <v>จังหวัด</v>
-      </c>
-      <c r="H1" t="str">
-        <v>หมายเหตุ</v>
+        <v>ประเภทลูกค้า</v>
       </c>
     </row>
     <row r="2">
@@ -452,13 +444,7 @@
         <v>อีเมลติดต่อ</v>
       </c>
       <c r="F2" t="str">
-        <v>เลขที่/ถนน/แขวง/เขต</v>
-      </c>
-      <c r="G2" t="str">
-        <v>จังหวัด</v>
-      </c>
-      <c r="H2" t="str">
-        <v>หมายเหตุเพิ่มเติม</v>
+        <v>DEVELOPER / ENDUSER / ผู้รับเหมา</v>
       </c>
     </row>
     <row r="3">
@@ -478,13 +464,7 @@
         <v>somchai@ncp.co.th</v>
       </c>
       <c r="F3" t="str">
-        <v>123 ถ.สีลม</v>
-      </c>
-      <c r="G3" t="str">
-        <v>กรุงเทพฯ</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
+        <v>DEVELOPER</v>
       </c>
     </row>
     <row r="4">
@@ -504,18 +484,32 @@
         <v/>
       </c>
       <c r="F4" t="str">
+        <v>ENDUSER</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>บริษัท รับเหมาก่อสร้าง</v>
+      </c>
+      <c r="B5" t="str">
+        <v>คุณมานะ แข็งแกร่ง</v>
+      </c>
+      <c r="C5" t="str">
         <v/>
       </c>
-      <c r="G4" t="str">
-        <v>กรุงเทพฯ</v>
-      </c>
-      <c r="H4" t="str">
-        <v>ลูกค้าประจำ</v>
+      <c r="D5" t="str">
+        <v>091-000-0000</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>ผู้รับเหมา</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>